<commit_message>
pipeline-projection: source real Base_MidLevel_Stock, answer H2
Base_MidLevel_Stock was the last placeholder input. Replaced it with the
real weighted mid-level headcount for Graphic Designers (IPUMS CPS,
OCC 2634, employed, age 26-35, 2022). Re-ran the independent verification
with all five inputs real; the gap magnitudes are unchanged from the
placeholder run, which corrects an earlier wrong claim that they weren't
meaningful yet (the stock anchor cancels out of Gap[t,s,N] by
construction, so Pass 2's gap numbers were already correct).

Updates H2's brief bracket from provisional to confirmed with the real
onset years and gap sizes at both training lags.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G369nNnTi7y8arxwb5saeB
</commit_message>
<xml_diff>
--- a/capabilities/pipeline-projection/model.xlsx
+++ b/capabilities/pipeline-projection/model.xlsx
@@ -803,11 +803,11 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>500</v>
+        <v>98685</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER. Actual or assumed mid-level headcount in Base_Year; same across all scenarios since none have diverged yet.</t>
+          <t>IPUMS CPS Basic Monthly, OCC 2634 (Graphic Designers), employed (EMPSTAT 10/12), age 26-35, 2022. Weighted headcount averaged across the 12 monthly samples (range 77,280-117,161; unweighted N=350 across the year, ~23-68/month). See prompt-log.md 2026-10-09 entry.</t>
         </is>
       </c>
     </row>

</xml_diff>